<commit_message>
Ajout de la Modelisation Merise dans le projet Latex
</commit_message>
<xml_diff>
--- a/Doc/FEUILLES DES DONNEES/FEUILLE DES DONNEES.xlsx
+++ b/Doc/FEUILLES DES DONNEES/FEUILLE DES DONNEES.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\musha\OneDrive\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projet\BAC3\Doc\FEUILLES DES DONNEES\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B73C1A9-9B55-42F6-9C9E-6E82D5CB2B4B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9888C65-4BD1-49B5-8EF1-27422774FB77}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12650" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12650" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="NOEUDS" sheetId="1" r:id="rId1"/>

</xml_diff>